<commit_message>
V2.0.15 + V2.0.16 + testes nas 17 empresas
</commit_message>
<xml_diff>
--- a/V. 2 (Pudim)/MODELO/dados_teste/RESULTADOS TESTES COMPARATIVOS.xlsx
+++ b/V. 2 (Pudim)/MODELO/dados_teste/RESULTADOS TESTES COMPARATIVOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ferna\dev_linux\FinScore\V. 2 (Pudim)\MODELO\dados_teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96B862AD-25A7-41C3-BB05-1E1B5123E2F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67AA3770-FBBE-4B7A-B6AA-ADA6D8CD8D39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{4010788E-9D57-4518-8E30-3FC23E7ECB45}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
   <si>
     <t>SIMULAÇÕES FINSCORE</t>
   </si>
@@ -164,23 +164,20 @@
     <t>FP</t>
   </si>
   <si>
-    <t>não roda: Residual negativo em p_Passivo_Circulante; a base deveria ter sido bloqueada</t>
-  </si>
-  <si>
-    <t>não roda: motivo desconhecido.</t>
-  </si>
-  <si>
     <t>PUDIM (V2.00.07)</t>
   </si>
   <si>
     <t>PUDIM (V2.00.12)</t>
+  </si>
+  <si>
+    <t>PUDIM (V2.00.15)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -192,14 +189,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -227,7 +216,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -249,6 +238,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -306,7 +301,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -323,9 +318,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
@@ -357,28 +349,49 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -2004,7 +2017,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93FCEEB7-B92B-4053-9C51-209D00D628B8}">
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
@@ -2016,54 +2029,68 @@
     <col min="7" max="8" width="13.88671875" style="1" customWidth="1"/>
     <col min="9" max="9" width="24.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="11" width="13.88671875" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="1"/>
+    <col min="12" max="12" width="24.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="13.88671875" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="F2" s="1" t="s">
         <v>38</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>38</v>
       </c>
+      <c r="L2" s="1" t="s">
+        <v>38</v>
+      </c>
     </row>
-    <row r="3" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="15" t="s">
+    <row r="3" spans="1:14" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="17" t="s">
+      <c r="C3" s="15"/>
+      <c r="D3" s="16" t="s">
         <v>36</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="J3" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="K3" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="L3" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="M3" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="H3" s="18" t="s">
+      <c r="N3" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="I3" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="J3" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="K3" s="21" t="s">
-        <v>40</v>
-      </c>
     </row>
-    <row r="4" spans="1:12" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="13">
+    <row r="4" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A4" s="12">
         <v>1</v>
       </c>
       <c r="B4" s="5" t="s">
@@ -2073,33 +2100,42 @@
         <f t="shared" ref="C4:C20" si="0">_xlfn.CONCAT(A4,RIGHT(B4,30))</f>
         <v>1Callamarys</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="13" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="5">
         <v>240</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="7">
         <v>401.22</v>
       </c>
-      <c r="G4" s="19">
+      <c r="G4" s="18">
         <v>572.29</v>
       </c>
-      <c r="H4" s="19">
+      <c r="H4" s="18">
         <v>332.11</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I4" s="10">
         <v>394.43</v>
       </c>
-      <c r="J4" s="22">
+      <c r="J4" s="21">
         <v>629.49</v>
       </c>
-      <c r="K4" s="22">
+      <c r="K4" s="21">
         <v>291.85000000000002</v>
       </c>
+      <c r="L4" s="27">
+        <v>412.23</v>
+      </c>
+      <c r="M4" s="28">
+        <v>564.25</v>
+      </c>
+      <c r="N4" s="28">
+        <v>338.27</v>
+      </c>
     </row>
-    <row r="5" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="13">
+    <row r="5" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="12">
         <v>2</v>
       </c>
       <c r="B5" s="5" t="s">
@@ -2109,33 +2145,36 @@
         <f t="shared" si="0"/>
         <v>2Cool Seed</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="13" t="s">
         <v>26</v>
       </c>
       <c r="E5" s="5">
         <v>392.5</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="8">
         <v>644.94000000000005</v>
       </c>
-      <c r="G5" s="20">
+      <c r="G5" s="19">
         <v>639.71</v>
       </c>
-      <c r="H5" s="20">
+      <c r="H5" s="19">
         <v>652.44000000000005</v>
       </c>
-      <c r="I5" s="12">
+      <c r="I5" s="11">
         <v>731.87</v>
       </c>
-      <c r="J5" s="23">
+      <c r="J5" s="22">
         <v>726.36</v>
       </c>
-      <c r="K5" s="23">
+      <c r="K5" s="22">
         <v>741.14</v>
       </c>
+      <c r="L5" s="29"/>
+      <c r="M5" s="30"/>
+      <c r="N5" s="30"/>
     </row>
-    <row r="6" spans="1:12" ht="72" x14ac:dyDescent="0.3">
-      <c r="A6" s="13">
+    <row r="6" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A6" s="12">
         <v>3</v>
       </c>
       <c r="B6" s="5" t="s">
@@ -2145,33 +2184,36 @@
         <f t="shared" si="0"/>
         <v>3 Cofesa - Super G Supermercado</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="13" t="s">
         <v>24</v>
       </c>
       <c r="E6" s="5">
         <v>200</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="8">
         <v>649.04</v>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="19">
         <v>585.73</v>
       </c>
-      <c r="H6" s="20">
+      <c r="H6" s="19">
         <v>748.18</v>
       </c>
-      <c r="I6" s="12">
+      <c r="I6" s="11">
         <v>726.56</v>
       </c>
-      <c r="J6" s="23">
+      <c r="J6" s="22">
         <v>647.85</v>
       </c>
-      <c r="K6" s="23">
+      <c r="K6" s="22">
         <v>874.75</v>
       </c>
+      <c r="L6" s="29"/>
+      <c r="M6" s="30"/>
+      <c r="N6" s="30"/>
     </row>
-    <row r="7" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="13">
+    <row r="7" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A7" s="12">
         <v>4</v>
       </c>
       <c r="B7" s="5" t="s">
@@ -2181,33 +2223,36 @@
         <f t="shared" si="0"/>
         <v>4t - E-Construmarket Tecnologia</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="13" t="s">
         <v>30</v>
       </c>
       <c r="E7" s="5">
         <v>650</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="8">
         <v>666.28</v>
       </c>
-      <c r="G7" s="20">
+      <c r="G7" s="19">
         <v>624.88</v>
       </c>
-      <c r="H7" s="20">
+      <c r="H7" s="19">
         <v>728.84</v>
       </c>
-      <c r="I7" s="12">
+      <c r="I7" s="11">
         <v>747.93</v>
       </c>
-      <c r="J7" s="23">
+      <c r="J7" s="22">
         <v>705.02</v>
       </c>
-      <c r="K7" s="23">
+      <c r="K7" s="22">
         <v>824.09</v>
       </c>
+      <c r="L7" s="29"/>
+      <c r="M7" s="30"/>
+      <c r="N7" s="30"/>
     </row>
-    <row r="8" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="13">
+    <row r="8" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="12">
         <v>5</v>
       </c>
       <c r="B8" s="5" t="s">
@@ -2217,33 +2262,36 @@
         <f t="shared" si="0"/>
         <v>5umarket - Mobicloud Tecnologia</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="13" t="s">
         <v>31</v>
       </c>
       <c r="E8" s="5">
         <v>905</v>
       </c>
-      <c r="F8" s="9">
+      <c r="F8" s="8">
         <v>766.21</v>
       </c>
-      <c r="G8" s="20">
+      <c r="G8" s="19">
         <v>785</v>
       </c>
-      <c r="H8" s="20">
+      <c r="H8" s="19">
         <v>758.54</v>
       </c>
-      <c r="I8" s="12">
+      <c r="I8" s="11">
         <v>897.64</v>
       </c>
-      <c r="J8" s="23">
+      <c r="J8" s="22">
         <v>927.28</v>
       </c>
-      <c r="K8" s="23">
+      <c r="K8" s="22">
         <v>883.03</v>
       </c>
+      <c r="L8" s="29"/>
+      <c r="M8" s="30"/>
+      <c r="N8" s="30"/>
     </row>
-    <row r="9" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="13">
+    <row r="9" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="12">
         <v>6</v>
       </c>
       <c r="B9" s="5" t="s">
@@ -2253,33 +2301,36 @@
         <f t="shared" si="0"/>
         <v>6strumarket - SSA-Miro Solucoes</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="13" t="s">
         <v>32</v>
       </c>
       <c r="E9" s="5">
         <v>255</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="8">
         <v>481.89</v>
       </c>
-      <c r="G9" s="20">
+      <c r="G9" s="19">
         <v>394.89</v>
       </c>
-      <c r="H9" s="20">
+      <c r="H9" s="19">
         <v>630.73</v>
       </c>
-      <c r="I9" s="12">
+      <c r="I9" s="11">
         <v>500</v>
       </c>
-      <c r="J9" s="23">
+      <c r="J9" s="22">
         <v>435.65</v>
       </c>
-      <c r="K9" s="23">
+      <c r="K9" s="22">
         <v>734.35</v>
       </c>
+      <c r="L9" s="29"/>
+      <c r="M9" s="30"/>
+      <c r="N9" s="30"/>
     </row>
-    <row r="10" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="13">
+    <row r="10" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="12">
         <v>7</v>
       </c>
       <c r="B10" s="5" t="s">
@@ -2289,36 +2340,36 @@
         <f t="shared" si="0"/>
         <v>7ornax - Flammers Participacoes</v>
       </c>
-      <c r="D10" s="14" t="s">
+      <c r="D10" s="13" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="5">
         <v>475</v>
       </c>
-      <c r="F10" s="24">
+      <c r="F10" s="23">
         <v>0</v>
       </c>
-      <c r="G10" s="24">
+      <c r="G10" s="23">
         <v>0</v>
       </c>
-      <c r="H10" s="24">
+      <c r="H10" s="23">
         <v>0</v>
       </c>
-      <c r="I10" s="25">
+      <c r="I10" s="24">
         <v>0</v>
       </c>
-      <c r="J10" s="25">
+      <c r="J10" s="24">
         <v>0</v>
       </c>
-      <c r="K10" s="25">
+      <c r="K10" s="24">
         <v>0</v>
       </c>
-      <c r="L10" s="6" t="s">
-        <v>42</v>
-      </c>
+      <c r="L10" s="31"/>
+      <c r="M10" s="31"/>
+      <c r="N10" s="31"/>
     </row>
-    <row r="11" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="13">
+    <row r="11" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A11" s="12">
         <v>8</v>
       </c>
       <c r="B11" s="5" t="s">
@@ -2328,33 +2379,36 @@
         <f t="shared" si="0"/>
         <v>8po Fornax - Fornax Consultoria</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="13" t="s">
         <v>18</v>
       </c>
       <c r="E11" s="5">
         <v>227.5</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="8">
         <v>737.56</v>
       </c>
-      <c r="G11" s="20">
+      <c r="G11" s="19">
         <v>809.47</v>
       </c>
-      <c r="H11" s="20">
+      <c r="H11" s="19">
         <v>715.79</v>
       </c>
-      <c r="I11" s="12">
+      <c r="I11" s="11">
         <v>854.01</v>
       </c>
-      <c r="J11" s="23">
+      <c r="J11" s="22">
         <v>961.69</v>
       </c>
-      <c r="K11" s="23">
+      <c r="K11" s="22">
         <v>808.95</v>
       </c>
+      <c r="L11" s="29"/>
+      <c r="M11" s="30"/>
+      <c r="N11" s="30"/>
     </row>
-    <row r="12" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="13">
+    <row r="12" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="12">
         <v>9</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -2364,33 +2418,36 @@
         <f t="shared" si="0"/>
         <v>9rupo Fornax - Modo Serviços RH</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="13" t="s">
         <v>21</v>
       </c>
       <c r="E12" s="5">
         <v>790</v>
       </c>
-      <c r="F12" s="9">
+      <c r="F12" s="8">
         <v>350</v>
       </c>
-      <c r="G12" s="20">
+      <c r="G12" s="19">
         <v>825.62</v>
       </c>
-      <c r="H12" s="20">
+      <c r="H12" s="19">
         <v>295.19</v>
       </c>
-      <c r="I12" s="12">
+      <c r="I12" s="11">
         <v>350</v>
       </c>
-      <c r="J12" s="23">
+      <c r="J12" s="22">
         <v>925</v>
       </c>
-      <c r="K12" s="23">
+      <c r="K12" s="22">
         <v>221.58</v>
       </c>
+      <c r="L12" s="29"/>
+      <c r="M12" s="30"/>
+      <c r="N12" s="30"/>
     </row>
-    <row r="13" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="13">
+    <row r="13" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="12">
         <v>10</v>
       </c>
       <c r="B13" s="5" t="s">
@@ -2400,33 +2457,36 @@
         <f t="shared" si="0"/>
         <v>10upo Fornax - Mooven Assessoria</v>
       </c>
-      <c r="D13" s="14" t="s">
+      <c r="D13" s="13" t="s">
         <v>20</v>
       </c>
       <c r="E13" s="5">
         <v>902.5</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="8">
         <v>249.87</v>
       </c>
-      <c r="G13" s="20">
+      <c r="G13" s="19">
         <v>428.95</v>
       </c>
-      <c r="H13" s="20">
+      <c r="H13" s="19">
         <v>190.55</v>
       </c>
-      <c r="I13" s="12">
+      <c r="I13" s="11">
         <v>244.87</v>
       </c>
-      <c r="J13" s="23">
+      <c r="J13" s="22">
         <v>443.16</v>
       </c>
-      <c r="K13" s="23">
+      <c r="K13" s="22">
         <v>170.46</v>
       </c>
+      <c r="L13" s="29"/>
+      <c r="M13" s="30"/>
+      <c r="N13" s="30"/>
     </row>
-    <row r="14" spans="1:12" ht="72" x14ac:dyDescent="0.3">
-      <c r="A14" s="13">
+    <row r="14" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A14" s="12">
         <v>11</v>
       </c>
       <c r="B14" s="5" t="s">
@@ -2436,33 +2496,36 @@
         <f t="shared" si="0"/>
         <v>11Grupo JNP - JNH Hoteis</v>
       </c>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="13" t="s">
         <v>22</v>
       </c>
       <c r="E14" s="5">
         <v>767.5</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F14" s="8">
         <v>532.41</v>
       </c>
-      <c r="G14" s="20">
+      <c r="G14" s="19">
         <v>747.52</v>
       </c>
-      <c r="H14" s="20">
+      <c r="H14" s="19">
         <v>454.01</v>
       </c>
-      <c r="I14" s="12">
+      <c r="I14" s="11">
         <v>602.53</v>
       </c>
-      <c r="J14" s="23">
+      <c r="J14" s="22">
         <v>875.11</v>
       </c>
-      <c r="K14" s="23">
+      <c r="K14" s="22">
         <v>486.21</v>
       </c>
+      <c r="L14" s="29"/>
+      <c r="M14" s="30"/>
+      <c r="N14" s="30"/>
     </row>
-    <row r="15" spans="1:12" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A15" s="13">
+    <row r="15" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="12">
         <v>12</v>
       </c>
       <c r="B15" s="5" t="s">
@@ -2472,33 +2535,36 @@
         <f t="shared" si="0"/>
         <v>12Grupo JNP - JNS Seguradora</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="D15" s="13" t="s">
         <v>23</v>
       </c>
       <c r="E15" s="5">
         <v>587.5</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F15" s="8">
         <v>390.38</v>
       </c>
-      <c r="G15" s="20">
+      <c r="G15" s="19">
         <v>373.08</v>
       </c>
-      <c r="H15" s="20">
+      <c r="H15" s="19">
         <v>416.08</v>
       </c>
-      <c r="I15" s="12">
+      <c r="I15" s="11">
         <v>376.14</v>
       </c>
-      <c r="J15" s="23">
+      <c r="J15" s="22">
         <v>356</v>
       </c>
-      <c r="K15" s="23">
+      <c r="K15" s="22">
         <v>411.72</v>
       </c>
+      <c r="L15" s="29"/>
+      <c r="M15" s="30"/>
+      <c r="N15" s="30"/>
     </row>
-    <row r="16" spans="1:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="13">
+    <row r="16" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A16" s="12">
         <v>13</v>
       </c>
       <c r="B16" s="5" t="s">
@@ -2508,33 +2574,36 @@
         <f t="shared" si="0"/>
         <v>13 - Mega Administradora de Bens</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="D16" s="13" t="s">
         <v>28</v>
       </c>
       <c r="E16" s="5">
         <v>157.5</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="8">
         <v>732.81</v>
       </c>
-      <c r="G16" s="20">
+      <c r="G16" s="19">
         <v>720.04</v>
       </c>
-      <c r="H16" s="20">
+      <c r="H16" s="19">
         <v>751.29</v>
       </c>
-      <c r="I16" s="12">
+      <c r="I16" s="11">
         <v>845.81</v>
       </c>
-      <c r="J16" s="23">
+      <c r="J16" s="22">
         <v>836.2</v>
       </c>
-      <c r="K16" s="23">
+      <c r="K16" s="22">
         <v>862.02</v>
       </c>
+      <c r="L16" s="29"/>
+      <c r="M16" s="30"/>
+      <c r="N16" s="30"/>
     </row>
-    <row r="17" spans="1:12" ht="72" x14ac:dyDescent="0.3">
-      <c r="A17" s="13">
+    <row r="17" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+      <c r="A17" s="12">
         <v>14</v>
       </c>
       <c r="B17" s="5" t="s">
@@ -2544,33 +2613,36 @@
         <f t="shared" si="0"/>
         <v>14Motos - Mega Motos Com Imp Exp</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="D17" s="13" t="s">
         <v>27</v>
       </c>
       <c r="E17" s="5">
         <v>847.5</v>
       </c>
-      <c r="F17" s="9">
+      <c r="F17" s="8">
         <v>560.29</v>
       </c>
-      <c r="G17" s="20">
+      <c r="G17" s="19">
         <v>623.65</v>
       </c>
-      <c r="H17" s="20">
+      <c r="H17" s="19">
         <v>530.13</v>
       </c>
-      <c r="I17" s="12">
+      <c r="I17" s="11">
         <v>621.24</v>
       </c>
-      <c r="J17" s="23">
+      <c r="J17" s="22">
         <v>701.43</v>
       </c>
-      <c r="K17" s="23">
+      <c r="K17" s="22">
         <v>576.78</v>
       </c>
+      <c r="L17" s="29"/>
+      <c r="M17" s="30"/>
+      <c r="N17" s="30"/>
     </row>
-    <row r="18" spans="1:12" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="13">
+    <row r="18" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A18" s="12">
         <v>15</v>
       </c>
       <c r="B18" s="5" t="s">
@@ -2580,36 +2652,36 @@
         <f t="shared" si="0"/>
         <v>15Log Road Transporte Rodoviario</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="13" t="s">
         <v>34</v>
       </c>
       <c r="E18" s="5">
         <v>717.5</v>
       </c>
-      <c r="F18" s="24">
+      <c r="F18" s="23">
         <v>0</v>
       </c>
-      <c r="G18" s="24">
+      <c r="G18" s="23">
         <v>0</v>
       </c>
-      <c r="H18" s="24">
+      <c r="H18" s="23">
         <v>0</v>
       </c>
-      <c r="I18" s="25">
+      <c r="I18" s="24">
         <v>0</v>
       </c>
-      <c r="J18" s="25">
+      <c r="J18" s="24">
         <v>0</v>
       </c>
-      <c r="K18" s="25">
+      <c r="K18" s="24">
         <v>0</v>
       </c>
-      <c r="L18" s="6" t="s">
-        <v>41</v>
-      </c>
+      <c r="L18" s="31"/>
+      <c r="M18" s="31"/>
+      <c r="N18" s="31"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A19" s="13">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A19" s="12">
         <v>16</v>
       </c>
       <c r="B19" s="5" t="s">
@@ -2619,33 +2691,36 @@
         <f t="shared" si="0"/>
         <v>16og Road - TMDL Armazens Gerais</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="13" t="s">
         <v>33</v>
       </c>
       <c r="E19" s="5">
         <v>295</v>
       </c>
-      <c r="F19" s="9">
+      <c r="F19" s="8">
         <v>752.8</v>
       </c>
-      <c r="G19" s="20">
+      <c r="G19" s="19">
         <v>829.87</v>
       </c>
-      <c r="H19" s="20">
+      <c r="H19" s="19">
         <v>716.04</v>
       </c>
-      <c r="I19" s="12">
+      <c r="I19" s="11">
         <v>837.55</v>
       </c>
-      <c r="J19" s="23">
+      <c r="J19" s="22">
         <v>989.67</v>
       </c>
-      <c r="K19" s="23">
+      <c r="K19" s="22">
         <v>755.72</v>
       </c>
+      <c r="L19" s="29"/>
+      <c r="M19" s="30"/>
+      <c r="N19" s="30"/>
     </row>
-    <row r="20" spans="1:12" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A20" s="13">
+    <row r="20" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="12">
         <v>17</v>
       </c>
       <c r="B20" s="5" t="s">
@@ -2655,30 +2730,33 @@
         <f t="shared" si="0"/>
         <v>17Pacto Energia</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="13" t="s">
         <v>29</v>
       </c>
       <c r="E20" s="5">
         <v>855</v>
       </c>
-      <c r="F20" s="9">
+      <c r="F20" s="8">
         <v>312.61</v>
       </c>
-      <c r="G20" s="20">
+      <c r="G20" s="19">
         <v>271.17</v>
       </c>
-      <c r="H20" s="20">
+      <c r="H20" s="19">
         <v>385.63</v>
       </c>
-      <c r="I20" s="12">
+      <c r="I20" s="11">
         <v>289.87</v>
       </c>
-      <c r="J20" s="23">
+      <c r="J20" s="22">
         <v>245.52</v>
       </c>
-      <c r="K20" s="23">
+      <c r="K20" s="22">
         <v>397.45</v>
       </c>
+      <c r="L20" s="29"/>
+      <c r="M20" s="30"/>
+      <c r="N20" s="30"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
V2.0.19 + testes / criticas elpidio (prints e comentarios whatsapp)
</commit_message>
<xml_diff>
--- a/V. 2 (Pudim)/MODELO/dados_teste/RESULTADOS TESTES COMPARATIVOS.xlsx
+++ b/V. 2 (Pudim)/MODELO/dados_teste/RESULTADOS TESTES COMPARATIVOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ferna\dev_linux\FinScore\V. 2 (Pudim)\MODELO\dados_teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67AA3770-FBBE-4B7A-B6AA-ADA6D8CD8D39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D060F96A-8508-40C7-991F-F4412A9EEE1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{4010788E-9D57-4518-8E30-3FC23E7ECB45}"/>
   </bookViews>
@@ -38,6 +38,44 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={F23ACFC9-4275-47DE-9335-6124AA9BE172}</author>
+  </authors>
+  <commentList>
+    <comment ref="L10" authorId="0" shapeId="0" xr:uid="{F23ACFC9-4275-47DE-9335-6124AA9BE172}">
+      <text>
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+Comentário:
+    ---------------------------------------------------------------------------
+RuntimeError                              Traceback (most recent call last)
+Cell In[332], line 14
+     10 diagnosticos_simulacao = {}
+     11 diagnosticos_simulacao_correlacionada = {}
+     12 
+     13 if MODELO_APTO:
+---&gt; 14     df_cenarios_deterministicos = run_deterministic_scenarios(
+     15         df_contas_analise, pca_observado
+     16     )
+     17     print("Cenários determinísticos:")
+Cell In[327], line 882, in run_deterministic_scenarios(base, profiles)
+    878     table["monotonicidade_global"] = monotonic
+    879     table["status_monotonicidade"] = "PASSOU" if monotonic else "FALHOU"
+    880     if not monotonic:
+    881         values = ordered_scores.to_dict() if not ordered_scores.empty else {}
+--&gt; 882         raise RuntimeError(
+    883             "Cenários não satisfazem Base &gt;= Adverso &gt;= Severo: "
+    884             f"{values}"
+    885         )
+RuntimeError: Cenários não satisfazem Base &gt;= Adverso &gt;= Severo: {'BASE': nan, 'ADVERSO': nan, 'SEVERO': nan}</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
   <si>
@@ -167,17 +205,17 @@
     <t>PUDIM (V2.00.07)</t>
   </si>
   <si>
-    <t>PUDIM (V2.00.12)</t>
-  </si>
-  <si>
-    <t>PUDIM (V2.00.15)</t>
+    <t>PUDIM (V2.00.19)</t>
+  </si>
+  <si>
+    <t>PUDIM (V2.00.13)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -214,6 +252,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -757,7 +801,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>PUDIM (V2.00.12)</c:v>
+                  <c:v>PUDIM (V2.00.13)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1700,6 +1744,12 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Fernando Vieira" id="{3BDFCCA5-60B3-42E1-B98C-617BAB224F75}" userId="f97fb756bfb044a9" providerId="Windows Live"/>
+</personList>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
   <a:themeElements>
@@ -2015,8 +2065,36 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="L10" dT="2026-08-13T20:38:12.06" personId="{3BDFCCA5-60B3-42E1-B98C-617BAB224F75}" id="{F23ACFC9-4275-47DE-9335-6124AA9BE172}">
+    <text>---------------------------------------------------------------------------
+RuntimeError                              Traceback (most recent call last)
+Cell In[332], line 14
+     10 diagnosticos_simulacao = {}
+     11 diagnosticos_simulacao_correlacionada = {}
+     12 
+     13 if MODELO_APTO:
+---&gt; 14     df_cenarios_deterministicos = run_deterministic_scenarios(
+     15         df_contas_analise, pca_observado
+     16     )
+     17     print("Cenários determinísticos:")
+Cell In[327], line 882, in run_deterministic_scenarios(base, profiles)
+    878     table["monotonicidade_global"] = monotonic
+    879     table["status_monotonicidade"] = "PASSOU" if monotonic else "FALHOU"
+    880     if not monotonic:
+    881         values = ordered_scores.to_dict() if not ordered_scores.empty else {}
+--&gt; 882         raise RuntimeError(
+    883             "Cenários não satisfazem Base &gt;= Adverso &gt;= Severo: "
+    884             f"{values}"
+    885         )
+RuntimeError: Cenários não satisfazem Base &gt;= Adverso &gt;= Severo: {'BASE': nan, 'ADVERSO': nan, 'SEVERO': nan}</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93FCEEB7-B92B-4053-9C51-209D00D628B8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93FCEEB7-B92B-4053-9C51-209D00D628B8}">
   <dimension ref="A1:N20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2071,7 +2149,7 @@
         <v>40</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J3" s="20" t="s">
         <v>39</v>
@@ -2080,7 +2158,7 @@
         <v>40</v>
       </c>
       <c r="L3" s="25" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M3" s="26" t="s">
         <v>39</v>
@@ -2169,9 +2247,15 @@
       <c r="K5" s="22">
         <v>741.14</v>
       </c>
-      <c r="L5" s="29"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="30"/>
+      <c r="L5" s="29">
+        <v>660.52</v>
+      </c>
+      <c r="M5" s="30">
+        <v>665.04</v>
+      </c>
+      <c r="N5" s="30">
+        <v>657.82</v>
+      </c>
     </row>
     <row r="6" spans="1:14" ht="72" x14ac:dyDescent="0.3">
       <c r="A6" s="12">
@@ -2208,9 +2292,15 @@
       <c r="K6" s="22">
         <v>874.75</v>
       </c>
-      <c r="L6" s="29"/>
-      <c r="M6" s="30"/>
-      <c r="N6" s="30"/>
+      <c r="L6" s="29">
+        <v>740.46</v>
+      </c>
+      <c r="M6" s="30">
+        <v>672.9</v>
+      </c>
+      <c r="N6" s="30">
+        <v>865.12</v>
+      </c>
     </row>
     <row r="7" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A7" s="12">
@@ -2247,9 +2337,15 @@
       <c r="K7" s="22">
         <v>824.09</v>
       </c>
-      <c r="L7" s="29"/>
-      <c r="M7" s="30"/>
-      <c r="N7" s="30"/>
+      <c r="L7" s="29">
+        <v>747.73</v>
+      </c>
+      <c r="M7" s="30">
+        <v>709.66</v>
+      </c>
+      <c r="N7" s="30">
+        <v>814.8</v>
+      </c>
     </row>
     <row r="8" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A8" s="12">
@@ -2286,9 +2382,15 @@
       <c r="K8" s="22">
         <v>883.03</v>
       </c>
-      <c r="L8" s="29"/>
-      <c r="M8" s="30"/>
-      <c r="N8" s="30"/>
+      <c r="L8" s="29">
+        <v>868.78</v>
+      </c>
+      <c r="M8" s="30">
+        <v>914.86</v>
+      </c>
+      <c r="N8" s="30">
+        <v>848.89</v>
+      </c>
     </row>
     <row r="9" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A9" s="12">
@@ -2325,9 +2427,15 @@
       <c r="K9" s="22">
         <v>734.35</v>
       </c>
-      <c r="L9" s="29"/>
-      <c r="M9" s="30"/>
-      <c r="N9" s="30"/>
+      <c r="L9" s="29">
+        <v>500</v>
+      </c>
+      <c r="M9" s="30">
+        <v>443.68</v>
+      </c>
+      <c r="N9" s="30">
+        <v>657.68</v>
+      </c>
     </row>
     <row r="10" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A10" s="12">
@@ -2364,9 +2472,15 @@
       <c r="K10" s="24">
         <v>0</v>
       </c>
-      <c r="L10" s="31"/>
-      <c r="M10" s="31"/>
-      <c r="N10" s="31"/>
+      <c r="L10" s="31">
+        <v>0</v>
+      </c>
+      <c r="M10" s="31">
+        <v>0</v>
+      </c>
+      <c r="N10" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A11" s="12">
@@ -2403,9 +2517,15 @@
       <c r="K11" s="22">
         <v>808.95</v>
       </c>
-      <c r="L11" s="29"/>
-      <c r="M11" s="30"/>
-      <c r="N11" s="30"/>
+      <c r="L11" s="29">
+        <v>809.48</v>
+      </c>
+      <c r="M11" s="30">
+        <v>971.24</v>
+      </c>
+      <c r="N11" s="30">
+        <v>744.69</v>
+      </c>
     </row>
     <row r="12" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A12" s="12">
@@ -2442,9 +2562,15 @@
       <c r="K12" s="22">
         <v>221.58</v>
       </c>
-      <c r="L12" s="29"/>
-      <c r="M12" s="30"/>
-      <c r="N12" s="30"/>
+      <c r="L12" s="29">
+        <v>350</v>
+      </c>
+      <c r="M12" s="30">
+        <v>916.67</v>
+      </c>
+      <c r="N12" s="30">
+        <v>295.26</v>
+      </c>
     </row>
     <row r="13" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A13" s="12">
@@ -2481,9 +2607,15 @@
       <c r="K13" s="22">
         <v>170.46</v>
       </c>
-      <c r="L13" s="29"/>
-      <c r="M13" s="30"/>
-      <c r="N13" s="30"/>
+      <c r="L13" s="29">
+        <v>303.26</v>
+      </c>
+      <c r="M13" s="30">
+        <v>469.6</v>
+      </c>
+      <c r="N13" s="30">
+        <v>230.78</v>
+      </c>
     </row>
     <row r="14" spans="1:14" ht="72" x14ac:dyDescent="0.3">
       <c r="A14" s="12">
@@ -2520,9 +2652,15 @@
       <c r="K14" s="22">
         <v>486.21</v>
       </c>
-      <c r="L14" s="29"/>
-      <c r="M14" s="30"/>
-      <c r="N14" s="30"/>
+      <c r="L14" s="29">
+        <v>647.52</v>
+      </c>
+      <c r="M14" s="30">
+        <v>874.86</v>
+      </c>
+      <c r="N14" s="30">
+        <v>549.03</v>
+      </c>
     </row>
     <row r="15" spans="1:14" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A15" s="12">
@@ -2559,9 +2697,15 @@
       <c r="K15" s="22">
         <v>411.72</v>
       </c>
-      <c r="L15" s="29"/>
-      <c r="M15" s="30"/>
-      <c r="N15" s="30"/>
+      <c r="L15" s="29">
+        <v>372.22</v>
+      </c>
+      <c r="M15" s="30">
+        <v>333.25</v>
+      </c>
+      <c r="N15" s="30">
+        <v>445.27</v>
+      </c>
     </row>
     <row r="16" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A16" s="12">
@@ -2598,9 +2742,15 @@
       <c r="K16" s="22">
         <v>862.02</v>
       </c>
-      <c r="L16" s="29"/>
-      <c r="M16" s="30"/>
-      <c r="N16" s="30"/>
+      <c r="L16" s="29">
+        <v>787.68</v>
+      </c>
+      <c r="M16" s="30">
+        <v>780.15</v>
+      </c>
+      <c r="N16" s="30">
+        <v>800.36</v>
+      </c>
     </row>
     <row r="17" spans="1:14" ht="72" x14ac:dyDescent="0.3">
       <c r="A17" s="12">
@@ -2637,9 +2787,15 @@
       <c r="K17" s="22">
         <v>576.78</v>
       </c>
-      <c r="L17" s="29"/>
-      <c r="M17" s="30"/>
-      <c r="N17" s="30"/>
+      <c r="L17" s="29">
+        <v>596.05999999999995</v>
+      </c>
+      <c r="M17" s="30">
+        <v>687.49</v>
+      </c>
+      <c r="N17" s="30">
+        <v>546.07000000000005</v>
+      </c>
     </row>
     <row r="18" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A18" s="12">
@@ -2676,9 +2832,15 @@
       <c r="K18" s="24">
         <v>0</v>
       </c>
-      <c r="L18" s="31"/>
-      <c r="M18" s="31"/>
-      <c r="N18" s="31"/>
+      <c r="L18" s="31">
+        <v>0</v>
+      </c>
+      <c r="M18" s="31">
+        <v>0</v>
+      </c>
+      <c r="N18" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="12">
@@ -2715,9 +2877,15 @@
       <c r="K19" s="22">
         <v>755.72</v>
       </c>
-      <c r="L19" s="29"/>
-      <c r="M19" s="30"/>
-      <c r="N19" s="30"/>
+      <c r="L19" s="29">
+        <v>813.9</v>
+      </c>
+      <c r="M19" s="30">
+        <v>984.4</v>
+      </c>
+      <c r="N19" s="30">
+        <v>728.59</v>
+      </c>
     </row>
     <row r="20" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A20" s="12">
@@ -2754,13 +2922,20 @@
       <c r="K20" s="22">
         <v>397.45</v>
       </c>
-      <c r="L20" s="29"/>
-      <c r="M20" s="30"/>
-      <c r="N20" s="30"/>
+      <c r="L20" s="29">
+        <v>307.89</v>
+      </c>
+      <c r="M20" s="30">
+        <v>250.22</v>
+      </c>
+      <c r="N20" s="30">
+        <v>432.62</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
revisão modelo v2.19 + implementação v2.19 no app
</commit_message>
<xml_diff>
--- a/V. 2 (Pudim)/MODELO/dados_teste/RESULTADOS TESTES COMPARATIVOS.xlsx
+++ b/V. 2 (Pudim)/MODELO/dados_teste/RESULTADOS TESTES COMPARATIVOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ferna\dev_linux\FinScore\V. 2 (Pudim)\MODELO\dados_teste\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D060F96A-8508-40C7-991F-F4412A9EEE1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DC6C761-1A96-4C24-9127-F4EB04A32B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{4010788E-9D57-4518-8E30-3FC23E7ECB45}"/>
   </bookViews>
@@ -42,6 +42,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={F23ACFC9-4275-47DE-9335-6124AA9BE172}</author>
+    <author>tc={133EC99E-66A0-4A77-8437-7486C9DCDDD8}</author>
   </authors>
   <commentList>
     <comment ref="L10" authorId="0" shapeId="0" xr:uid="{F23ACFC9-4275-47DE-9335-6124AA9BE172}">
@@ -70,6 +71,53 @@
     884             f"{values}"
     885         )
 RuntimeError: Cenários não satisfazem Base &gt;= Adverso &gt;= Severo: {'BASE': nan, 'ADVERSO': nan, 'SEVERO': nan}</t>
+      </text>
+    </comment>
+    <comment ref="L18" authorId="1" shapeId="0" xr:uid="{133EC99E-66A0-4A77-8437-7486C9DCDDD8}">
+      <text>
+        <t xml:space="preserve">[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+Comentário:
+    ---------------------------------------------------------------------------
+ValueError                                Traceback (most recent call last)
+Cell In[705], line 22
+     18     display(df_cenarios_deterministicos.round(4))
+     19     if NUM_SIMULACOES &lt; 100:
+     20         raise ValueError("Use ao menos 100 simulações.")
+     21 
+---&gt; 22     df_simulacoes_independentes, diagnosticos_simulacao = run_sensitivity(
+     23         df_contas_analise, NUM_SIMULACOES, SEMENTE,
+     24         pca_observado, "independente",
+     25     )
+Cell In[700], line 580, in run_sensitivity(base, n, seed, profiles, approach)
+    576     rows, rejected_rows, flag_counts = [], [], {}
+    577     attempts = 0
+    578     while len(rows) &lt; n and attempts &lt; n * MAX_ATTEMPT_FACTOR:
+    579         attempts += 1
+--&gt; 580         sim = simulate_trajectory(base, widths, rng, approach)
+    581         flags = accounting_flags(sim)
+    582         characteristics = _relative_shocks(base, sim)
+    583         characteristics.update({
+Cell In[700], line 355, in simulate_trajectory(base, widths, rng, approach)
+    351         sim, base, "p_Ativo_Circulante",
+    352         ["p_Caixa_Equivalentes", "p_Contas_Receber_Clientes", "p_Estoques"],
+    353         widths["p_Ativo_Circulante"], factors["p_Ativo_Circulante"],
+    354     )
+--&gt; 355     _rebuild_total(
+    356         sim, base, "p_Passivo_Circulante",
+    357         [
+    358             "p_Fornecedores", "p_Obrigacoes_Tributarias_CP",
+Cell In[700], line 115, in _rebuild_total(sim, base, total, parts, width, factor)
+    111             base.loc[rebuild, total]
+    112             - base.loc[rebuild, parts].sum(axis=1, skipna=True)
+    113         ).to_numpy(float)
+    114         if (residual &lt; -1e-9).any():
+--&gt; 115             raise ValueError(f"Residual negativo em {total}.")
+    116         residual_sim = _sample_nonnegative(
+    117             np.maximum(residual, 0.0), width, factor[rebuild.to_numpy()]
+    118         )
+ValueError: Residual negativo em p_Passivo_Circulante.
+</t>
       </text>
     </comment>
   </commentList>
@@ -2090,6 +2138,48 @@
     885         )
 RuntimeError: Cenários não satisfazem Base &gt;= Adverso &gt;= Severo: {'BASE': nan, 'ADVERSO': nan, 'SEVERO': nan}</text>
   </threadedComment>
+  <threadedComment ref="L18" dT="2026-08-14T00:10:11.13" personId="{3BDFCCA5-60B3-42E1-B98C-617BAB224F75}" id="{133EC99E-66A0-4A77-8437-7486C9DCDDD8}">
+    <text xml:space="preserve">---------------------------------------------------------------------------
+ValueError                                Traceback (most recent call last)
+Cell In[705], line 22
+     18     display(df_cenarios_deterministicos.round(4))
+     19     if NUM_SIMULACOES &lt; 100:
+     20         raise ValueError("Use ao menos 100 simulações.")
+     21 
+---&gt; 22     df_simulacoes_independentes, diagnosticos_simulacao = run_sensitivity(
+     23         df_contas_analise, NUM_SIMULACOES, SEMENTE,
+     24         pca_observado, "independente",
+     25     )
+Cell In[700], line 580, in run_sensitivity(base, n, seed, profiles, approach)
+    576     rows, rejected_rows, flag_counts = [], [], {}
+    577     attempts = 0
+    578     while len(rows) &lt; n and attempts &lt; n * MAX_ATTEMPT_FACTOR:
+    579         attempts += 1
+--&gt; 580         sim = simulate_trajectory(base, widths, rng, approach)
+    581         flags = accounting_flags(sim)
+    582         characteristics = _relative_shocks(base, sim)
+    583         characteristics.update({
+Cell In[700], line 355, in simulate_trajectory(base, widths, rng, approach)
+    351         sim, base, "p_Ativo_Circulante",
+    352         ["p_Caixa_Equivalentes", "p_Contas_Receber_Clientes", "p_Estoques"],
+    353         widths["p_Ativo_Circulante"], factors["p_Ativo_Circulante"],
+    354     )
+--&gt; 355     _rebuild_total(
+    356         sim, base, "p_Passivo_Circulante",
+    357         [
+    358             "p_Fornecedores", "p_Obrigacoes_Tributarias_CP",
+Cell In[700], line 115, in _rebuild_total(sim, base, total, parts, width, factor)
+    111             base.loc[rebuild, total]
+    112             - base.loc[rebuild, parts].sum(axis=1, skipna=True)
+    113         ).to_numpy(float)
+    114         if (residual &lt; -1e-9).any():
+--&gt; 115             raise ValueError(f"Residual negativo em {total}.")
+    116         residual_sim = _sample_nonnegative(
+    117             np.maximum(residual, 0.0), width, factor[rebuild.to_numpy()]
+    118         )
+ValueError: Residual negativo em p_Passivo_Circulante.
+</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 

</xml_diff>